<commit_message>
Deployed bb27427 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Premiere/nsi_premiere.xlsx
+++ b/NSI_Premiere/nsi_premiere.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Premiere\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{6E4EF43E-DACA-465A-91A7-2E60A589D7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270CCDE7-958E-44C6-B7F9-65A560DC14FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="5" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" firstSheet="1" activeTab="5" xr2:uid="{C3D69442-6D2C-43E5-8165-E9BA2FDD5BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -21,10 +21,9 @@
     <sheet name="Feuil6" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Feuil6!$A$1:$G$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Feuil6!$A$1:$G$89</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="396">
   <si>
     <r>
       <t>ThèmeContenus (Compétence)Capacités attendues &amp; CommentairesN° Activité</t>
@@ -1454,6 +1453,96 @@
   <si>
     <t>Fait</t>
   </si>
+  <si>
+    <t>RD01_Cours</t>
+  </si>
+  <si>
+    <t>RD01_Synth</t>
+  </si>
+  <si>
+    <t>RD01_ACT1</t>
+  </si>
+  <si>
+    <t>RD01_EXO1</t>
+  </si>
+  <si>
+    <t>RD01_EXO2</t>
+  </si>
+  <si>
+    <t>RD01_EXO3</t>
+  </si>
+  <si>
+    <t>RD01_EXO4</t>
+  </si>
+  <si>
+    <t>RD01_flashcard</t>
+  </si>
+  <si>
+    <t>RD01_quiz</t>
+  </si>
+  <si>
+    <t>Algebre Boole</t>
+  </si>
+  <si>
+    <t>RD02_Cours</t>
+  </si>
+  <si>
+    <t>RD02_Synth</t>
+  </si>
+  <si>
+    <t>RD02_EXO1</t>
+  </si>
+  <si>
+    <t>RD02_EXO2</t>
+  </si>
+  <si>
+    <t>Circuit logique</t>
+  </si>
+  <si>
+    <t>RD03_Cours</t>
+  </si>
+  <si>
+    <t>RD03_Synth</t>
+  </si>
+  <si>
+    <t>RD03_EXO1</t>
+  </si>
+  <si>
+    <t>RD03_ACT1</t>
+  </si>
+  <si>
+    <t>Flottants</t>
+  </si>
+  <si>
+    <t>RD04_Cours</t>
+  </si>
+  <si>
+    <t>Texte</t>
+  </si>
+  <si>
+    <t>RD05_Cours</t>
+  </si>
+  <si>
+    <t>RD05_ACT1</t>
+  </si>
+  <si>
+    <t>RD06</t>
+  </si>
+  <si>
+    <t>Donnees en Table</t>
+  </si>
+  <si>
+    <t>RD06_Cours</t>
+  </si>
+  <si>
+    <t>RD06_ACT1</t>
+  </si>
+  <si>
+    <t>ARSE01_ACT1</t>
+  </si>
+  <si>
+    <t>Assembleur</t>
+  </si>
 </sst>
 </file>
 
@@ -1496,7 +1585,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1524,6 +1613,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1555,7 +1650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1580,6 +1675,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3773,7 +3869,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27B06C93-FCDE-4C7C-B0AD-5832CC1D02CA}">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.265625" style="8" customWidth="1"/>
@@ -5243,7 +5339,9 @@
       <c r="G68" s="9"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A69" s="10"/>
+      <c r="A69" s="10" t="s">
+        <v>173</v>
+      </c>
       <c r="B69" s="10" t="s">
         <v>323</v>
       </c>
@@ -5262,7 +5360,9 @@
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A70" s="10"/>
+      <c r="A70" s="10" t="s">
+        <v>173</v>
+      </c>
       <c r="B70" s="10" t="s">
         <v>323</v>
       </c>
@@ -5270,32 +5370,34 @@
         <v>324</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>228</v>
+        <v>211</v>
       </c>
       <c r="E70" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F70" s="10" t="s">
-        <v>326</v>
-      </c>
-      <c r="G70" s="10"/>
+        <v>394</v>
+      </c>
+      <c r="G70" s="10" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A71" s="10"/>
       <c r="B71" s="10" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F71" s="10" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="G71" s="10"/>
     </row>
@@ -5308,13 +5410,13 @@
         <v>328</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E72" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F72" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G72" s="10"/>
     </row>
@@ -5327,13 +5429,13 @@
         <v>328</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>331</v>
+        <v>226</v>
       </c>
       <c r="F73" s="10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G73" s="10"/>
     </row>
@@ -5352,30 +5454,30 @@
         <v>331</v>
       </c>
       <c r="F74" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="G74" s="10" t="s">
-        <v>260</v>
-      </c>
+        <v>332</v>
+      </c>
+      <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A75" s="10"/>
       <c r="B75" s="10" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>226</v>
+        <v>331</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>335</v>
-      </c>
-      <c r="G75" s="10"/>
+        <v>333</v>
+      </c>
+      <c r="G75" s="10" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A76" s="10"/>
@@ -5386,13 +5488,13 @@
         <v>334</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E76" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F76" s="10" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G76" s="10"/>
     </row>
@@ -5405,13 +5507,13 @@
         <v>334</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>331</v>
+        <v>226</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="G77" s="10"/>
     </row>
@@ -5430,35 +5532,35 @@
         <v>331</v>
       </c>
       <c r="F78" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="G78" s="10"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A79" s="10"/>
+      <c r="B79" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="E79" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="F79" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="G78" s="10" t="s">
+      <c r="G79" s="10" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A79" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="B79" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="F79" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="G79" s="10"/>
-    </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A80" s="10"/>
+      <c r="A80" s="10" t="s">
+        <v>173</v>
+      </c>
       <c r="B80" s="10" t="s">
         <v>340</v>
       </c>
@@ -5466,39 +5568,39 @@
         <v>341</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E80" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F80" s="10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G80" s="10"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A81" s="10" t="s">
-        <v>173</v>
-      </c>
+      <c r="A81" s="10"/>
       <c r="B81" s="10" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F81" s="10" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="G81" s="10"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A82" s="10"/>
+      <c r="A82" s="10" t="s">
+        <v>173</v>
+      </c>
       <c r="B82" s="10" t="s">
         <v>344</v>
       </c>
@@ -5506,13 +5608,13 @@
         <v>345</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E82" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F82" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G82" s="10"/>
     </row>
@@ -5525,20 +5627,18 @@
         <v>345</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G83" s="10"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A84" s="10" t="s">
-        <v>173</v>
-      </c>
+      <c r="A84" s="10"/>
       <c r="B84" s="10" t="s">
         <v>344</v>
       </c>
@@ -5546,13 +5646,13 @@
         <v>345</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E84" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F84" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G84" s="10"/>
     </row>
@@ -5561,19 +5661,19 @@
         <v>173</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="G85" s="10"/>
     </row>
@@ -5588,41 +5688,43 @@
         <v>351</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E86" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F86" s="10" t="s">
-        <v>352</v>
-      </c>
-      <c r="G86" s="10" t="s">
-        <v>353</v>
-      </c>
+        <v>354</v>
+      </c>
+      <c r="G86" s="10"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A87" s="10" t="s">
         <v>173</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F87" s="10" t="s">
-        <v>357</v>
-      </c>
-      <c r="G87" s="10"/>
+        <v>352</v>
+      </c>
+      <c r="G87" s="10" t="s">
+        <v>353</v>
+      </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A88" s="10"/>
+      <c r="A88" s="10" t="s">
+        <v>173</v>
+      </c>
       <c r="B88" s="10" t="s">
         <v>355</v>
       </c>
@@ -5630,20 +5732,507 @@
         <v>356</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E88" s="10" t="s">
         <v>226</v>
       </c>
       <c r="F88" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="G88" s="10"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A89" s="10"/>
+      <c r="B89" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="C89" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="D89" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="E89" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="F89" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="G88" s="10" t="s">
+      <c r="G89" s="10" t="s">
         <v>359</v>
       </c>
     </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A90" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B90" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E90" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F90" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="G90" s="12"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A91" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C91" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="E91" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F91" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="G91" s="12"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A92" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B92" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D92" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="E92" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F92" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="G92" s="12"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A93" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B93" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E93" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F93" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="G93" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A94" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B94" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D94" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E94" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F94" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="G94" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A95" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B95" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C95" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E95" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F95" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="G95" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A96" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B96" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E96" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="G96" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A97" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B97" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C97" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D97" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E97" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F97" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="G97" s="12"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A98" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B98" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D98" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E98" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F98" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="G98" s="12"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A99" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B99" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="D99" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E99" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F99" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="G99" s="12"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A100" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B100" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="D100" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="E100" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F100" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="G100" s="12"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A101" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B101" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C101" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="D101" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E101" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F101" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="G101" s="12"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A102" s="12"/>
+      <c r="B102" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C102" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="D102" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E102" s="12"/>
+      <c r="F102" s="12" t="s">
+        <v>379</v>
+      </c>
+      <c r="G102" s="12" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A103" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B103" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C103" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E103" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F103" s="12" t="s">
+        <v>381</v>
+      </c>
+      <c r="G103" s="12"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A104" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B104" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C104" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="E104" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F104" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="G104" s="12"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A105" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B105" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C105" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D105" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="E105" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F105" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="G105" s="12"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A106" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B106" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C106" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D106" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="E106" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F106" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="G106" s="12"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A107" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B107" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="C107" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="D107" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E107" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F107" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="G107" s="12"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A108" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B108" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C108" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="D108" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E108" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F108" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="G108" s="12"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A109" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B109" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="D109" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="E109" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F109" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="G109" s="12"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A110" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B110" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="D110" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="E110" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F110" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="G110" s="12"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A111" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B111" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="C111" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="D111" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="E111" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F111" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="G111" s="12"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G88" xr:uid="{27B06C93-FCDE-4C7C-B0AD-5832CC1D02CA}"/>
+  <autoFilter ref="A1:G89" xr:uid="{27B06C93-FCDE-4C7C-B0AD-5832CC1D02CA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>